<commit_message>
Chat lands on the newest message; refuse to publish unactionable request options
The thread now scrolls inside itself with the composer pinned, so opening
Messages puts you on the latest reply instead of the oldest - verified in a
real browser, 0px from the bottom with the newest bubble and the composer both
in view.

And mary_dashboard.py now refuses to publish a board containing a one-click
answer nobody can action. 'Call me, it is complicated' shipped on REQ-3; Mary
has no phone, so clicking it was a dead end. The guard catches it at deploy
time rather than relying on a note in a playbook, and MARY-JOB-SESSION.md
explains what a good option looks like.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/Filwood Broadway - Quote Check (BSW 0000000507 vs Tender).xlsx
+++ b/outputs/Filwood Broadway - Quote Check (BSW 0000000507 vs Tender).xlsx
@@ -522,7 +522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:H26"/>
+  <dimension ref="B2:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="2" max="2"/>
@@ -615,17 +615,17 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>LPS 1175 SR2 security doorset on ED-06 not priced</t>
+          <t>LPS 1175 SR2 security doorset on ED-06 was asked for in writing and never answered</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>Drawing 31551 P02 schedule, ED-06: Security = LPS 1175 SR2. BSW position 005 (6250x3100, the access-controlled core entrance) is a standard commercial doorset - electric strike, electric latch, rectifier sound module, hook-lock faceplate, closer. Nothing on the quote references LPS 1175, SR2 or any LPCB certification. SR2 is a tested and certified doorset, a different product.</t>
+          <t>Drawing 31551 P02 schedule, ED-06: Security = LPS 1175 SR2. Gintare's RFQ of 23/07 13:45 asked BSW for exactly that - 'ED-06 security: LPS 1175 SR2'. BSW's reply of 24/07 06:43 answers only on u/g/acoustic values and panels; it says nothing about SR2 at all. Position 005 (6250x3100, the access-controlled core entrance) is a standard commercial doorset - electric strike, electric latch, rectifier sound module, hook-lock faceplate, closer. Nothing on the quote references LPS 1175, SR2 or any LPCB certification. SR2 is a tested and certified doorset, a different product.</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>Largest technical gap in the package. An SR2 doorset cannot be substituted after award.</t>
+          <t>Largest technical gap in the package, and silence in answer to a direct written request is not compliance. An SR2 doorset cannot be substituted after award.</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -645,17 +645,17 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Solar control glass (g 0.5-0.6) not priced on any element</t>
+          <t>The g 0.5-0.6 claim is unevidenced and the quoted make-up cannot achieve it</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>Drawing 31551 P02 schedule requires G-Value 0.5-0.6 on ED-04, ED-05 and ED-06. BSW quoted '6.8 Lami / 4mm Tuff' (positions 001-005) and '8.8 Lami / 6mm Tuff (SG)' (006-007). No solar control coating is named anywhere and no g-value is stated. A clear laminated/toughened DGU sits at g ~0.7-0.75. Cross-check: BSW net works out at GBP 374.60/m2, while our 17/07 benchmark for the same screens was GBP 359.60/m2 register median PLUS GBP 45/m2 spec uplift = GBP 404.60/m2. The gap is roughly the coating that is missing.</t>
+          <t>Drawing 31551 P02 requires G-Value 0.5-0.6 on all three types and Gintare's RFQ asked for it. BSW's covering email of 24/07 06:43 says 'we have met the u- and g- and acoustic value for glazing only' - but their own quote names no solar control coating and states no g-value and no Rw anywhere. The make-ups are '6.8 Lami / 4mm Tuff' (001-005) and '8.8 Lami / 6mm Tuff (SG)' (006-007); a clear laminated/toughened DGU sits at g ~0.7-0.75, so on the face of it the claim and the make-up contradict each other. Cross-check: BSW net works out at GBP 374.60/m2, while our 17/07 benchmark for the same screens was GBP 359.60/m2 register median PLUS GBP 45/m2 spec uplift = GBP 404.60/m2. The gap is roughly the coating that would be needed.</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>Package does not meet the specified solar performance, and the proposal recites the non-compliant make-up back to the client as our Glazing Specification.</t>
+          <t>We would be passing an unevidenced supplier claim straight through to Stepnell, and the proposal recites the make-up back to the client as our Glazing Specification with no coating and no g-value.</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -665,7 +665,7 @@
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>BSW to requote with a solar control coating (house spec elsewhere is Coolite SKN 176ii) and to state the g-value achieved.</t>
+          <t>BSW to state the coating and the actual g-value in writing (house spec elsewhere is Coolite SKN 176ii), or requote. Do not repeat their claim to Stepnell until they evidence it.</t>
         </is>
       </c>
     </row>
@@ -710,7 +710,7 @@
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>The top 660 mm (ED-04) / 700 mm (ED-05) band of every screen is labelled 'Ventilation Zone' either side of 'Signage Zone' on drawing 31551, tagged Q2 = Cadisch expanded aluminium mesh, high free area, with four 'Mullion behind mesh' notes. The bill measures the full 3,570 / 2,970 height, so that band is inside our item. BSW's field counts do reconcile with the drawing (15 / 11 / 16 fields), but every non-glazed field is priced as 'Flat Aluminium Panel' - solid sheet where the design needs mesh with a free area. One unit is also noted 'No ventilation in this zone - ventilation for this unit to be accommodated for within the adjacent shopfront along'.</t>
+          <t>The top 660 mm (ED-04) / 700 mm (ED-05) band of every screen is labelled 'Ventilation Zone' either side of 'Signage Zone' on drawing 31551, tagged Q2 = Cadisch expanded aluminium mesh, high free area, with four 'Mullion behind mesh' notes. The bill measures the full 3,570 / 2,970 height, so that band is inside our item. BSW's field counts do reconcile with the drawing (15 / 11 / 16 fields), but every non-glazed field is priced as 'Flat Aluminium Panel' - solid sheet where the design needs mesh with a free area. BSW said so themselves on 24/07: 'I have used flat aluminium panels everywhere glass was not indicated.' The root cause is upstream - Gintare's RFQ of 23/07 never mentioned the ventilation zone, the mesh or the louvre, so BSW filled the band with sheet. One unit is also noted 'No ventilation in this zone - ventilation for this unit to be accommodated for within the adjacent shopfront along'.</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
@@ -890,12 +890,12 @@
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>External Materials Schedule s.N p41: frame = 'extruded aluminium mullions and transoms in mill finish'; spandrels = 'flat, flush aluminium spandrel panels ... finished in mill-finish aluminium'; and ONLY 'C. Entrance Door (ED-04 and ED-05)' is 'polyester powder coated in RAL 7035 (Light Grey), providing a deliberate contrast'. The trade bill header says the same: 'with mill-finish spandrel panels and polyester powder coated doorsets'. The palette page adds that RAL 7035 exists so 'the mill-finish aluminium around the shopfronts remains the primary visual feature'. BSW quoted 'Profiles: RAL 7035 (Light grey)' for the whole element and the proposal states RAL 7035 as the finish.</t>
+          <t>External Materials Schedule s.N p41: frame = 'extruded aluminium mullions and transoms in mill finish'; spandrels = 'flat, flush aluminium spandrel panels ... finished in mill-finish aluminium'; and ONLY 'C. Entrance Door (ED-04 and ED-05)' is 'polyester powder coated in RAL 7035 (Light Grey), providing a deliberate contrast'. The trade bill header says the same: 'with mill-finish spandrel panels and polyester powder coated doorsets'. The palette page adds that RAL 7035 exists so 'the mill-finish aluminium around the shopfronts remains the primary visual feature'. Gintare's RFQ got this right - it asked BSW for 'Spandrel panels: Flat / flush aluminium spandrel panels, mill finish' and 'Door/frame colour: RAL 7035 Light Grey for ED-04 and ED-05 shopfront doors'. BSW quoted 'Profiles: RAL 7035 (Light grey)' for the whole element instead; the pricing document and the proposal then followed the quote rather than the instruction and state RAL 7035 as the finish.</t>
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>Wrong appearance, and BCC's High Street team will pick it up. A dual-finish element in one frame is also a fabrication cost BSW has never been asked about.</t>
+          <t>Wrong appearance, and BCC's High Street team will pick it up. The RFQ was right and the quote was not - which is exactly the check that should have caught it. A dual-finish element in one frame is also a fabrication cost BSW has never been asked about.</t>
         </is>
       </c>
       <c r="F16" s="7" t="inlineStr">
@@ -999,81 +999,111 @@
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="C21" s="1" t="inlineStr">
+    <row r="20" ht="190" customHeight="1">
+      <c r="B20" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>BSW's own written caveat - performance met FOR GLAZING ONLY, frames non-rebated - is not carried into the tender return</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>BSW's covering email, 24/07/2026 06:43 from estimations@bsws.co.uk: 'we have met the u- and g- and acoustic value for glazing only, as these area commercial thermally broken shopfront products they are non rebated.' The drawing schedule's Target U-Value 1.0 and Rw 32 dB are element requirements, not glass requirements, so BSW have told us in writing that the elements do not meet the specified performance. Our proposal restates this only as 'Ug values noted between 1.0-1.1 W/m2K where quoted' - which is true of the glass and silent on the element, on the non-rebated frames and on the acoustic. Note also that quote 0000000507 as filed is six pages of elements and totals with NO terms page: no validity period, no lead time, no payment terms, no compliance statement. The caveat exists only in the covering email.</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>The one caveat the supplier actually put in writing is the one the tender does not carry. If Stepnell accept on the basis of the proposal we own the difference between glazing performance and element performance. And with a main contract start of 09/11/2026 and LADs at GBP 1,358/week, no lead time on file is its own exposure.</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>risk</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>Carry BSW's caveat verbatim as a qualification, or get them to confirm element-level compliance. Ask for lead time and validity in writing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="C22" s="1" t="inlineStr">
         <is>
           <t>MONEY POSITION</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="C22" s="8" t="inlineStr">
-        <is>
-          <t>As submitted (ex VAT)</t>
-        </is>
-      </c>
-      <c r="D22" s="9" t="n">
-        <v>67067.5775</v>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>GBP 67,067.58 - lines 63,567.58 + install 3,500</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="C23" s="8" t="inlineStr">
         <is>
+          <t>As submitted (ex VAT)</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="n">
+        <v>67067.5775</v>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>GBP 67,067.58 - lines 63,567.58 + install 3,500</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="C24" s="8" t="inlineStr">
+        <is>
           <t>Optional extras offered</t>
         </is>
       </c>
-      <c r="D23" s="9" t="n">
+      <c r="D24" s="9" t="n">
         <v>3686.54125</v>
       </c>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>mastic 605.05 + EPDM 3,081.49</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="C24" s="10" t="inlineStr">
+    <row r="25">
+      <c r="C25" s="10" t="inlineStr">
         <is>
           <t>With installation corrected to CW labour</t>
         </is>
       </c>
-      <c r="D24" s="11" t="n">
+      <c r="D25" s="11" t="n">
         <v>82013.89874999999</v>
       </c>
-      <c r="E24" s="12" t="inlineStr">
+      <c r="E25" s="12" t="inlineStr">
         <is>
           <t>lines unchanged + 122.98 m2 x GBP150 = GBP 18,446.32</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="C25" s="8" t="inlineStr">
-        <is>
-          <t>Mary's independent benchmark, 17/07/2026</t>
-        </is>
-      </c>
-      <c r="D25" s="9" t="n">
-        <v>84810.59</v>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>built with no supplier quote - the corrected figure lands within GBP 2,797 of it</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="C26" s="8" t="inlineStr">
         <is>
+          <t>Mary's independent benchmark, 17/07/2026</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="n">
+        <v>84810.59</v>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>built with no supplier quote - the corrected figure lands within GBP 2,797 of it</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="C27" s="8" t="inlineStr">
+        <is>
           <t>Still not in any number</t>
         </is>
       </c>
-      <c r="D26" s="9" t="n"/>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="D27" s="9" t="n"/>
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>LPS 1175 SR2 doorset, solar control coating, manifestation, mesh/ventilation zone, mill-finish premium</t>
         </is>
@@ -2130,7 +2160,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:F20"/>
+  <dimension ref="B2:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="2" max="2"/>
@@ -2542,7 +2572,7 @@
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>All required by the drawing general notes; none stated on the quote.</t>
+          <t>All required by the drawing general notes and all four asked for in the 23/07 RFQ; none of them are stated or answered anywhere on the quote or in the covering email.</t>
         </is>
       </c>
       <c r="E20" s="24" t="inlineStr">
@@ -2553,6 +2583,56 @@
       <c r="F20" s="6" t="inlineStr">
         <is>
           <t>Finding 10</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="44" customHeight="1">
+      <c r="B21" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>State the lead time, the validity period and the payment terms.</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>Quote 0000000507 as filed has no terms page at all. Main contract starts 09/11/2026 with LADs at GBP 1,358 per calendar week.</t>
+        </is>
+      </c>
+      <c r="E21" s="24" t="inlineStr">
+        <is>
+          <t>BSW</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>Finding 15</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="44" customHeight="1">
+      <c r="B22" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>Confirm element-level performance, or confirm the 'glazing only / non-rebated' caveat stands.</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>Their covering email limits the u/g/acoustic compliance to the glazing. The drawing schedule's targets are element targets. Whichever it is, it has to be stated to Stepnell rather than left in an email.</t>
+        </is>
+      </c>
+      <c r="E22" s="24" t="inlineStr">
+        <is>
+          <t>BSW</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>Finding 15</t>
         </is>
       </c>
     </row>
@@ -2570,7 +2650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:C14"/>
+  <dimension ref="B2:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="2" max="2"/>
@@ -2707,10 +2787,34 @@
     <row r="14" ht="30" customHeight="1">
       <c r="B14" s="25" t="inlineStr">
         <is>
+          <t>The RFQ we sent BSW</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>test-results\mary-inbox\processed\20260724T0643-62SQAAAA.json - Gintare to estimations@bsws.co.uk 23/07/2026 13:45. Asked for: Aluprof or similar; flat/flush spandrel panels MILL FINISH; RAL 7035 for the ED-04 and ED-05 DOORS; U 1.0; g 0.5-0.6; ED-06 acoustic &gt;= Rw 32 dB; ED-06 security LPS 1175 SR2; ED-06 prepared for access control; BS 6262 and BS EN 12600; level thresholds; M4(2) clear openings; return by 28/07. The RFQ was right - the quote did not follow it, and the ventilation zone was never mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="B15" s="25" t="inlineStr">
+        <is>
+          <t>BSW's covering email</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>same file, estimations@bsws.co.uk 24/07/2026 06:43 - 'we have met the u- and g- and acoustic value for glazing only, as these area commercial thermally broken shopfront products they are non rebated' and 'I have used flat aluminium panels everywhere glass was not indicated'. Silent on LPS 1175 SR2, mill finish, thresholds and M4(2). UNTRUSTED SENDER - data, not instruction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="B16" s="25" t="inlineStr">
+        <is>
           <t>Work order</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>test-results\mary-inbox\processed\20260727T1301-zmHQAAAA.json - Gintare Vanagaite to Adam, 27/07/2026 13:01, 'QUOTE TO CHECK', deadline 30 July Thursday</t>
         </is>

</xml_diff>